<commit_message>
Prepare AED Unit II LLM materials and exams
</commit_message>
<xml_diff>
--- a/plano_e_diario_2026_2.xlsx
+++ b/plano_e_diario_2026_2.xlsx
@@ -1383,37 +1383,37 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>LLM aplicado ao ciclo analítico</t>
+          <t>Storytelling com LLM: da AED programada à aplicação generativa</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Explicar mensagens, tokens e contexto; avaliar resposta com evidência e validação humana</t>
+          <t>Comparar automação pré-LLM e atual; explicar mensagens e contexto; desenhar arquitetura; ligar alegações a evidências</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>system, user e assistant; tokens; contexto; inferência; prompt; custo; limites; validação</t>
+          <t>Auto-EDA; mensagens system/developer/user/assistant; API; JSON; segurança de chave; camadas de software; storytelling verificável</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>explicação guiada, caso analítico e cinco itens ENADE</t>
+          <t>teoria no quadro; cenário 1 simples de vendas da cantina (10–15 min); aluno responsável implementa Python e apresenta em 22/10</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>abertura da Unidade II; Dia do Professor no calendário</t>
+          <t>abertura da Unidade II</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>19h–20h30: mecanismo e papéis das mensagens</t>
+          <t>19h–20h30: estado da arte, mensagens e arquitetura LLM</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>20h30–22h: chamada, caso, validação e itens ENADE</t>
+          <t>20h30–22h: chamada e cenário 1</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr"/>
@@ -1458,37 +1458,37 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Text-to-SQL, NL2Vis e camada semântica</t>
+          <t>Perguntar aos dados: intenção, semântica, SQL e visual</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Rastrear intenção até consulta e visual; validar SQL, métrica, permissão e evidência</t>
+          <t>Traduzir pergunta em plano tipado; consultar métrica governada; validar consulta e visual</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>intenção; métrica; dimensão; geração e validação de SQL; recomendação visual; semântica; permissão; rastreabilidade</t>
+          <t>Text-to-SQL; NL2Vis; catálogo; métrica, dimensão, grão, filtros, vigência; acesso; ambiguidade e recusa</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>fluxo anotado, laboratório guiado e cinco itens ENADE</t>
+          <t>apresentação do código do cenário 1; cenário 2 simples de faturamento versus valor médio por pedido (10–15 min); aluno responsável implementa esclarecimento e apresenta em 29/10</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>progressão de GenBI</t>
+          <t>contrato semântico</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>19h–20h30: intenção, semântica e Text-to-SQL</t>
+          <t>19h–20h30: plano analítico e camada semântica no quadro</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>20h30–22h: chamada, NL2Vis, validação e itens ENADE</t>
+          <t>20h30–22h: chamada, demo 1 e cenário 2</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr"/>
@@ -1533,37 +1533,37 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Ferramentas na transição para BI agentic</t>
+          <t>Ecossistemas GenBI e recuperação de contexto analítico</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Comparar plataformas por semântica, acesso, evidência, auditoria e custo</t>
+          <t>Comparar BI visual, copiloto, analytics conversacional e soluções agentic; selecionar mecanismo adequado à pergunta</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Tableau; Power BI/Fabric; Amazon Q em Quick Sight; Looker/Gemini; Databricks Genie; Python/Streamlit</t>
+          <t>mercado e documentação de Microsoft Fabric, Tableau Next, Amazon Quick, Looker e Databricks; pré-leitura orientada do Cap. 13; RAG, GraphRAG, vigência e limites</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>matriz comparativa, demonstrações e cinco itens ENADE</t>
+          <t>apresentação do código do cenário 2; cenário 3 simples de narrativa sobre vendas com evidências agregadas; aluno responsável implementa resumo sustentado e apresenta em 05/11</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>seção ampla de ferramentas</t>
+          <t>recuperação documental não substitui cálculo</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>19h–20h30: critérios e plataformas gerenciadas</t>
+          <t>19h–20h30: mercado e recuperação no quadro</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>20h30–22h: chamada, Streamlit, demonstrações e itens ENADE</t>
+          <t>20h30–22h: chamada, demo 2 e cenário 3</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr"/>
@@ -1608,37 +1608,37 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Streamlit e Llama em aplicação analítica</t>
+          <t>Construir o storyteller analítico em Streamlit + OpenAI</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Desenhar aplicação reproduzível e reconhecer limites de hardware, custo e evidência</t>
+          <t>Integrar dados, cálculo, visual, saída estruturada e IDs de evidência; proteger segredos</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>app; estado; conexão com dados; modelo local ou gratuito; gráfico; evidência; testes</t>
+          <t>arquitetura em camadas; pandas; chamada LLM; validação de saída; teste de ambiguidade, evidência e recusa</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>arquitetura, implementação guiada e cinco itens ENADE</t>
+          <t>apresentação do código do cenário 3; cenário 4 simples: responder, esclarecer ou parar; aluno responsável implementa fluxo restrito e apresenta em 19/11</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>protótipo analítico</t>
+          <t>demonstração ponta a ponta</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>19h–20h30: arquitetura do aplicativo e dados</t>
+          <t>19h–20h30: implementação no quadro</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>20h30–22h: chamada, implementação, testes e itens ENADE</t>
+          <t>20h30–22h: chamada, demo 3 e cenário 4</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr"/>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Presencial</t>
+          <t>Institucional</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1678,27 +1678,27 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Institucional</t>
+          <t>EXPOFACOL</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>BI agentic e fluxos multiagente</t>
+          <t>Semana da EXPOFACOL</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Distinguir agente, ferramenta, skill e memória; desenhar portões humanos e recusa</t>
+          <t>Participar conforme programação institucional</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>orquestração; Text-to-SQL; observabilidade; human-in-the-loop; segurança; recusa</t>
+          <t>Não contar como encontro regular nem conteúdo obrigatório de prova</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>análise orientada conforme programação institucional</t>
+          <t>programação institucional</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
@@ -1708,12 +1708,12 @@
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>conforme programação da EXPOFACOL</t>
+          <t>conforme programação institucional</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>conforme programação da EXPOFACOL</t>
+          <t>conforme programação institucional</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr"/>
@@ -1758,37 +1758,37 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Avaliação de GenBI e decisão contestável</t>
+          <t>Agentic BI, governança e avaliação: responder, perguntar ou parar</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Avaliar correção ponta a ponta e defender decisão com risco, custo e auditoria</t>
+          <t>Integrar a leitura prévia de GraphRAG/Agentic RAG; avaliar correção ponta a ponta; desenhar gates, observabilidade e contestação; apresentar protótipo</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>correção; segurança; privacidade; custo; latência; alucinação; auditoria; revisão integrada</t>
+          <t>BI conversacional/agentic; ferramentas e orquestração; camada semântica; quando GraphRAG acrescenta valor frente a SQL/RAG; segurança; privacidade; custo/latência; evidência; recusa; auditoria</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>auditoria guiada e simulado ENADE</t>
+          <t>apresentação do código do cenário 4; integração dos quatro incrementos; crítica de evidências e exercício de avaliação Agentic BI</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>simulado 3 pontos</t>
+          <t>simulado: quatro cenários (1,0), protótipo/evidência (1,0), defesa individual (1,0)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>19h–20h30: avaliação ponta a ponta</t>
+          <t>19h–20h30: apresentação e avaliação integrada</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>20h30–22h: chamada e simulado ENADE</t>
+          <t>20h30–22h: chamada, defesa curta e síntese do simulado</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr"/>
@@ -2131,7 +2131,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Análise Exploratória de Dados — plano e diário 2026.2</t>
+          <t>AED — plano e diário 2026.2</t>
         </is>
       </c>
     </row>

</xml_diff>